<commit_message>
chore: atualiza planilhas de Cadastro de Clientes e Clientes Especiais Hidracor
</commit_message>
<xml_diff>
--- a/public/Cadastro Clientes Hidracor.xlsx
+++ b/public/Cadastro Clientes Hidracor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\MIDAS RENT A CAR\midas-log\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A24098-76E0-4A1B-AD37-4B4865AAC5CE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2459560-F969-4490-85F7-C0CBECC14C8C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27524,9 +27524,6 @@
       <c r="D650" t="s">
         <v>2</v>
       </c>
-      <c r="E650" t="s">
-        <v>909</v>
-      </c>
     </row>
     <row r="651" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A651" t="s">
@@ -42862,7 +42859,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="1745" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1745" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1745" t="s">
         <v>5349</v>
       </c>
@@ -42876,7 +42873,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="1746" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1746" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1746" t="s">
         <v>125</v>
       </c>
@@ -42889,8 +42886,11 @@
       <c r="D1746" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="1747" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1746" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="1747" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1747" t="s">
         <v>5351</v>
       </c>
@@ -42904,7 +42904,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="1748" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1748" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1748" t="s">
         <v>654</v>
       </c>
@@ -42918,7 +42918,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="1749" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1749" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1749" t="s">
         <v>174</v>
       </c>
@@ -42932,7 +42932,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="1750" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1750" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1750" t="s">
         <v>2738</v>
       </c>
@@ -42946,7 +42946,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="1751" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1751" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1751" t="s">
         <v>5354</v>
       </c>
@@ -42960,7 +42960,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="1752" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1752" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1752" t="s">
         <v>5356</v>
       </c>
@@ -42974,7 +42974,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="1753" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1753" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1753" t="s">
         <v>2739</v>
       </c>
@@ -42988,7 +42988,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="1754" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1754" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1754" t="s">
         <v>2741</v>
       </c>
@@ -43002,7 +43002,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="1755" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1755" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1755" t="s">
         <v>5358</v>
       </c>
@@ -43016,7 +43016,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="1756" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1756" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1756" t="s">
         <v>4127</v>
       </c>
@@ -43030,7 +43030,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1757" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1757" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1757" t="s">
         <v>4129</v>
       </c>
@@ -43044,7 +43044,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="1758" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1758" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1758" t="s">
         <v>463</v>
       </c>
@@ -43058,7 +43058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="1759" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1759" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1759" t="s">
         <v>2744</v>
       </c>
@@ -43072,7 +43072,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="1760" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1760" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1760" t="s">
         <v>807</v>
       </c>

</xml_diff>